<commit_message>
Update safety incident data
</commit_message>
<xml_diff>
--- a/data/patnet_aichi_archive.xlsx
+++ b/data/patnet_aichi_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="incidents" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'incidents'!$A$1:$N$947</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'incidents'!$A$1:$N$948</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N947"/>
+  <dimension ref="A1:N948"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -64866,8 +64866,76 @@
         </is>
       </c>
     </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>d5a85209b9dbc24600d8</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>10月26日(月)午後3時15分頃</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>声かけ・不審者情報</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>不審者情報</t>
+        </is>
+      </c>
+      <c r="E948" t="inlineStr">
+        <is>
+          <t>犬山市</t>
+        </is>
+      </c>
+      <c r="F948" s="2" t="inlineStr">
+        <is>
+          <t>犬山市付近（地域代表点）</t>
+        </is>
+      </c>
+      <c r="G948" t="inlineStr">
+        <is>
+          <t>犬山市</t>
+        </is>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>municipality</t>
+        </is>
+      </c>
+      <c r="I948" t="n">
+        <v>35.378441</v>
+      </c>
+      <c r="J948" t="n">
+        <v>136.944427</v>
+      </c>
+      <c r="K948" s="3" t="inlineStr">
+        <is>
+          <t>声かけ・不審者情報に関する情報です。</t>
+        </is>
+      </c>
+      <c r="L948" s="3" t="inlineStr">
+        <is>
+          <t>2人組のうち1名の男が帰宅中の男子生徒に対して、「こっち来たらお菓子あげるよ」と声をかけた</t>
+        </is>
+      </c>
+      <c r="M948" s="4" t="inlineStr">
+        <is>
+          <t>http://patnet.jp/2026/10/26/%e7%8a%ac%e5%b1%b1%e5%b8%82-110/</t>
+        </is>
+      </c>
+      <c r="N948" t="inlineStr">
+        <is>
+          <t>2026-10-27T00:30:43+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N947"/>
+  <autoFilter ref="A1:N948"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -65815,6 +65883,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M945" r:id="rId944"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M946" r:id="rId945"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M947" r:id="rId946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M948" r:id="rId947"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>